<commit_message>
Update mock client data
</commit_message>
<xml_diff>
--- a/docs/sample-client-import.xlsx
+++ b/docs/sample-client-import.xlsx
@@ -163,11 +163,6 @@
           <t xml:space="preserve">drissa.nguessan@example.ci</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -240,11 +235,6 @@
           <t xml:space="preserve">nabintou.tanoh@example.ci</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -317,11 +307,6 @@
           <t xml:space="preserve">serge.cisse@example.ci</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -394,11 +379,6 @@
           <t xml:space="preserve">akissi.ouattara@example.ci</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -471,11 +451,6 @@
           <t xml:space="preserve">ahou.sangare@example.ci</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q6" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -548,11 +523,6 @@
           <t xml:space="preserve">amenan.traore@example.ci</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -625,11 +595,6 @@
           <t xml:space="preserve">patrice.seri@example.ci</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q8" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -687,11 +652,6 @@
           <t xml:space="preserve">contact@ivoireagroservices.ci</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -764,11 +724,6 @@
           <t xml:space="preserve">awa.traore@example.ci</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -841,11 +796,6 @@
           <t xml:space="preserve">adjoua.diallo@example.ci</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -918,11 +868,6 @@
           <t xml:space="preserve">seydou.camara@example.ci</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -995,11 +940,6 @@
           <t xml:space="preserve">nabintou.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1072,11 +1012,6 @@
           <t xml:space="preserve">aicha.sangare@example.ci</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -1149,11 +1084,6 @@
           <t xml:space="preserve">zie.seri@example.ci</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1211,11 +1141,6 @@
           <t xml:space="preserve">contact@batirensembleimmob.ci</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1288,11 +1213,6 @@
           <t xml:space="preserve">akissi.keita@example.ci</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1365,11 +1285,6 @@
           <t xml:space="preserve">felix.kone@example.ci</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q18" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -1442,11 +1357,6 @@
           <t xml:space="preserve">mamadou.cisse@example.ci</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1519,11 +1429,6 @@
           <t xml:space="preserve">prisca.camara@example.ci</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1596,11 +1501,6 @@
           <t xml:space="preserve">affoue.doumbia@example.ci</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q21" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -1673,11 +1573,6 @@
           <t xml:space="preserve">oumou.bakayoko@example.ci</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1750,11 +1645,6 @@
           <t xml:space="preserve">sylvie.tanoh@example.ci</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1827,11 +1717,6 @@
           <t xml:space="preserve">affoue.toure@example.ci</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1889,11 +1774,6 @@
           <t xml:space="preserve">contact@ongsantepourtous.ci</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -1966,11 +1846,6 @@
           <t xml:space="preserve">aicha.aka@example.ci</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2043,11 +1918,6 @@
           <t xml:space="preserve">affoue.coulibaly@example.ci</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2120,11 +1990,6 @@
           <t xml:space="preserve">bintou.bakayoko@example.ci</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q28" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2197,11 +2062,6 @@
           <t xml:space="preserve">aicha.yao@example.ci</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q29" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2274,11 +2134,6 @@
           <t xml:space="preserve">armand.nguessan@example.ci</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q30" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2351,11 +2206,6 @@
           <t xml:space="preserve">djeneba.kouame@example.ci</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2428,11 +2278,6 @@
           <t xml:space="preserve">sekou.bakayoko@example.ci</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2505,11 +2350,6 @@
           <t xml:space="preserve">zie.bakayoko@example.ci</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -2582,11 +2422,6 @@
           <t xml:space="preserve">assetou.diallo@example.ci</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q34" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -2659,11 +2494,6 @@
           <t xml:space="preserve">oumou.keita@example.ci</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2736,11 +2566,6 @@
           <t xml:space="preserve">amadou.sangare@example.ci</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2813,11 +2638,6 @@
           <t xml:space="preserve">patrice.diallo@example.ci</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2890,11 +2710,6 @@
           <t xml:space="preserve">ismael.oulai@example.ci</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -2967,11 +2782,6 @@
           <t xml:space="preserve">awa.cisse@example.ci</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q39" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3044,11 +2854,6 @@
           <t xml:space="preserve">rokia.fofana@example.ci</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -3106,11 +2911,6 @@
           <t xml:space="preserve">contact@associationespoirj.ci</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3183,11 +2983,6 @@
           <t xml:space="preserve">ismael.keita@example.ci</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q42" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3260,11 +3055,6 @@
           <t xml:space="preserve">adama.nguessan@example.ci</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q43" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3337,11 +3127,6 @@
           <t xml:space="preserve">vamara.fofana@example.ci</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q44" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3414,11 +3199,6 @@
           <t xml:space="preserve">koffi.toure@example.ci</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3491,11 +3271,6 @@
           <t xml:space="preserve">seydou.sangare@example.ci</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q46" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3568,11 +3343,6 @@
           <t xml:space="preserve">nadege.sangare@example.ci</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3645,11 +3415,6 @@
           <t xml:space="preserve">bakary.seri@example.ci</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q48" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3722,11 +3487,6 @@
           <t xml:space="preserve">oumou.sylla@example.ci</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3799,11 +3559,6 @@
           <t xml:space="preserve">nadege.fofana@example.ci</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q50" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -3876,11 +3631,6 @@
           <t xml:space="preserve">adjoua.toure@example.ci</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q51" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -3953,11 +3703,6 @@
           <t xml:space="preserve">korotoum.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q52" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4030,11 +3775,6 @@
           <t xml:space="preserve">oumou.seri@example.ci</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q53" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4107,11 +3847,6 @@
           <t xml:space="preserve">karim.ouattara@example.ci</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4184,11 +3919,6 @@
           <t xml:space="preserve">mariame.bamba@example.ci</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4261,11 +3991,6 @@
           <t xml:space="preserve">ahou.cisse@example.ci</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4338,11 +4063,6 @@
           <t xml:space="preserve">ibrahim.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4415,11 +4135,6 @@
           <t xml:space="preserve">adama.oulai@example.ci</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q58" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4477,11 +4192,6 @@
           <t xml:space="preserve">contact@atlantiquelogistiq.ci</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q59" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4554,11 +4264,6 @@
           <t xml:space="preserve">assetou.fofana@example.ci</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q60" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4631,11 +4336,6 @@
           <t xml:space="preserve">bakary.gnahore@example.ci</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q61" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4708,11 +4408,6 @@
           <t xml:space="preserve">nadege.koffi@example.ci</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q62" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -4785,11 +4480,6 @@
           <t xml:space="preserve">vamara.ouattara@example.ci</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q63" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4862,11 +4552,6 @@
           <t xml:space="preserve">adama.assi@example.ci</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -4939,11 +4624,6 @@
           <t xml:space="preserve">kadidja.sylla@example.ci</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q65" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -5016,11 +4696,6 @@
           <t xml:space="preserve">serge.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q66" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5093,11 +4768,6 @@
           <t xml:space="preserve">mariame.cisse@example.ci</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q67" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5155,11 +4825,6 @@
           <t xml:space="preserve">contact@groupementworodoug.ci</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q68" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5232,11 +4897,6 @@
           <t xml:space="preserve">affoue.bakayoko@example.ci</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q69" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5309,11 +4969,6 @@
           <t xml:space="preserve">moussa.kone@example.ci</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q70" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -5386,11 +5041,6 @@
           <t xml:space="preserve">mariame.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q71" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5463,11 +5113,6 @@
           <t xml:space="preserve">kouassi.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q72" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5540,11 +5185,6 @@
           <t xml:space="preserve">drissa.sylla@example.ci</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -5617,11 +5257,6 @@
           <t xml:space="preserve">mariam.camara@example.ci</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q74" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5694,11 +5329,6 @@
           <t xml:space="preserve">karim.fofana@example.ci</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q75" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -5771,11 +5401,6 @@
           <t xml:space="preserve">mamadou.konate@example.ci</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q76" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -5848,11 +5473,6 @@
           <t xml:space="preserve">kouadio.kouame@example.ci</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q77" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -5925,11 +5545,6 @@
           <t xml:space="preserve">serge.diabate@example.ci</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q78" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6002,11 +5617,6 @@
           <t xml:space="preserve">assetou.kouassi@example.ci</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6079,11 +5689,6 @@
           <t xml:space="preserve">aboubacar.toure@example.ci</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q80" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6156,11 +5761,6 @@
           <t xml:space="preserve">sylvie.traore@example.ci</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q81" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6233,11 +5833,6 @@
           <t xml:space="preserve">patrice.diabate@example.ci</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q82" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6310,11 +5905,6 @@
           <t xml:space="preserve">ibrahim.keita@example.ci</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q83" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6387,11 +5977,6 @@
           <t xml:space="preserve">affoue.nguessan@example.ci</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q84" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -6464,11 +6049,6 @@
           <t xml:space="preserve">awa.ouattara@example.ci</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q85" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6541,11 +6121,6 @@
           <t xml:space="preserve">armand.nguessan2@example.ci</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6618,11 +6193,6 @@
           <t xml:space="preserve">prisca.coulibaly2@example.ci</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6695,11 +6265,6 @@
           <t xml:space="preserve">prisca.coulibaly@example.ci</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
-        </is>
-      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6772,11 +6337,6 @@
           <t xml:space="preserve">nadege.yao@example.ci</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-COC</t>
-        </is>
-      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -6834,11 +6394,6 @@
           <t xml:space="preserve">contact@sankorenegoce.ci</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6896,11 +6451,6 @@
           <t xml:space="preserve">contact@cooperativekavokiv.ci</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q91" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -6973,11 +6523,6 @@
           <t xml:space="preserve">clarisse.seri@example.ci</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SPY-CTR</t>
-        </is>
-      </c>
       <c r="Q92" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -7050,11 +6595,6 @@
           <t xml:space="preserve">clarisse.brou@example.ci</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -7127,11 +6667,6 @@
           <t xml:space="preserve">nabintou.brou@example.ci</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q94" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -7204,11 +6739,6 @@
           <t xml:space="preserve">adama.diallo@example.ci</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YAM-CTR</t>
-        </is>
-      </c>
       <c r="Q95" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -7281,11 +6811,6 @@
           <t xml:space="preserve">sekou.assi@example.ci</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BKE-CTR</t>
-        </is>
-      </c>
       <c r="Q96" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -7358,11 +6883,6 @@
           <t xml:space="preserve">ahou.zadi@example.ci</t>
         </is>
       </c>
-      <c r="P97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q97" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -7435,11 +6955,6 @@
           <t xml:space="preserve">nadege.zadi@example.ci</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-PLT</t>
-        </is>
-      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t xml:space="preserve">fr</t>
@@ -7512,11 +7027,6 @@
           <t xml:space="preserve">seydou.keita@example.ci</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KHG-CTR</t>
-        </is>
-      </c>
       <c r="Q99" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -7589,11 +7099,6 @@
           <t xml:space="preserve">rokia.zadi@example.ci</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLA-CTR</t>
-        </is>
-      </c>
       <c r="Q100" t="inlineStr">
         <is>
           <t xml:space="preserve">en</t>
@@ -7664,11 +7169,6 @@
       <c r="O101" t="inlineStr">
         <is>
           <t xml:space="preserve">ibrahim.traore@example.ci</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ABJ-YOP</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">

</xml_diff>